<commit_message>
fixes the issue with blank columns
</commit_message>
<xml_diff>
--- a/tests/data/structural.bad-blank.xlsx
+++ b/tests/data/structural.bad-blank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Documents/nuh-helper/tests/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF4B5857-7388-F146-B2B8-13A6EDDE0703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DC7B6A-8930-5345-AAD3-D51733BA3AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1880" windowWidth="28040" windowHeight="17180" xr2:uid="{DE17C082-B7AC-184B-8DE6-41F02A2D59B3}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ptid</t>
   </si>
@@ -76,6 +76,18 @@
   </si>
   <si>
     <t>forbidden</t>
+  </si>
+  <si>
+    <t>cake</t>
+  </si>
+  <si>
+    <t>froot</t>
+  </si>
+  <si>
+    <t>nuh77</t>
+  </si>
+  <si>
+    <t>nuh78</t>
   </si>
 </sst>
 </file>
@@ -448,7 +460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC4D2730-B112-7747-9DD9-A971A0C530E0}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -496,6 +508,28 @@
       </c>
       <c r="D4" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="1">
+        <v>33865</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1">
+        <v>29110</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>